<commit_message>
chore: Update AI Champions Initiative Report.xlsx with latest data
</commit_message>
<xml_diff>
--- a/AI Champions Initiative Report.xlsx
+++ b/AI Champions Initiative Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mpi2cob\Boopathi\Repository\workspace_ai_champion_tracting_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83CC2F66-502C-4F3A-986C-03F7ABBE3779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9DE40A5-80BC-476F-8F62-E135E95F1CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D2E0B207-558B-4F0A-AA5E-53ABE0D8DD5B}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="75">
   <si>
     <t>Initiative Name</t>
   </si>
@@ -242,15 +242,6 @@
   </si>
   <si>
     <t>Phase 2 updates are in-progress</t>
-  </si>
-  <si>
-    <t>Repriortization is going on</t>
-  </si>
-  <si>
-    <t>Collect input from the team on the feedback of Claude</t>
-  </si>
-  <si>
-    <t>Get the information from central team as well</t>
   </si>
   <si>
     <r>
@@ -283,12 +274,39 @@
   <si>
     <t>Repository - Capture the information - AI topics Gen AI Stories</t>
   </si>
+  <si>
+    <t>Repriortization is going on - Sanjeev Sharma will be taking over this topic</t>
+  </si>
+  <si>
+    <r>
+      <t>Collect input from the team on the feedback of Claude, Get the information from central team as well -</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> We are not proceeding with this topic. </t>
+    </r>
+  </si>
+  <si>
+    <t>Pilot version</t>
+  </si>
+  <si>
+    <t>Deploy application in onRender tool</t>
+  </si>
+  <si>
+    <t>Dynamic sharepoint Integration</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -383,6 +401,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -723,7 +748,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -810,12 +835,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -828,7 +847,6 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -846,7 +864,19 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="13" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -870,12 +900,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -887,18 +911,25 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1262,7 +1293,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="77" t="s">
+      <c r="A2" s="56" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="1"/>
@@ -1275,7 +1306,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="77"/>
+      <c r="A3" s="56"/>
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1290,7 +1321,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="77"/>
+      <c r="A4" s="56"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="2" t="s">
@@ -1301,7 +1332,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="77"/>
+      <c r="A5" s="56"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="2" t="s">
@@ -1312,7 +1343,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="77"/>
+      <c r="A6" s="56"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2" t="s">
@@ -1323,7 +1354,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="78"/>
+      <c r="A7" s="57"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="5" t="s">
@@ -1361,7 +1392,7 @@
       <c r="B10" s="11"/>
       <c r="C10" s="12">
         <f>AVERAGE(C11:C25)</f>
-        <v>0.48571428571428571</v>
+        <v>0.47272727272727266</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="14"/>
@@ -1387,13 +1418,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="15"/>
-      <c r="B12" s="64" t="s">
+      <c r="B12" s="65" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="66">
+      <c r="C12" s="67">
         <v>0.5</v>
       </c>
-      <c r="D12" s="60" t="s">
+      <c r="D12" s="61" t="s">
         <v>27</v>
       </c>
       <c r="E12" s="33" t="s">
@@ -1403,27 +1434,27 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="15"/>
-      <c r="B13" s="65"/>
-      <c r="C13" s="67"/>
-      <c r="D13" s="68"/>
+      <c r="B13" s="66"/>
+      <c r="C13" s="68"/>
+      <c r="D13" s="69"/>
       <c r="E13" s="34" t="s">
         <v>66</v>
       </c>
       <c r="F13" s="16"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="15"/>
       <c r="B14" s="28" t="s">
         <v>31</v>
       </c>
       <c r="C14" s="29">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D14" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="31" t="s">
-        <v>67</v>
+      <c r="E14" s="76" t="s">
+        <v>70</v>
       </c>
       <c r="F14" s="16"/>
     </row>
@@ -1432,7 +1463,9 @@
       <c r="B15" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="35"/>
+      <c r="C15" s="29">
+        <v>0.3</v>
+      </c>
       <c r="D15" s="30" t="s">
         <v>14</v>
       </c>
@@ -1441,38 +1474,38 @@
       </c>
       <c r="F15" s="27"/>
     </row>
-    <row r="16" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="15"/>
-      <c r="B16" s="69" t="s">
+      <c r="B16" s="70" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="71"/>
-      <c r="D16" s="73" t="s">
+      <c r="C16" s="77">
+        <v>1</v>
+      </c>
+      <c r="D16" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="36" t="s">
-        <v>68</v>
-      </c>
-      <c r="F16" s="79">
-        <v>46325</v>
+      <c r="E16" s="79" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="58">
+        <v>46265</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="15"/>
-      <c r="B17" s="70"/>
-      <c r="C17" s="72"/>
-      <c r="D17" s="74"/>
-      <c r="E17" s="37" t="s">
-        <v>69</v>
-      </c>
-      <c r="F17" s="80"/>
+      <c r="B17" s="71"/>
+      <c r="C17" s="78"/>
+      <c r="D17" s="73"/>
+      <c r="E17" s="80"/>
+      <c r="F17" s="59"/>
     </row>
     <row r="18" spans="1:6" ht="27.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="15"/>
       <c r="B18" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="38">
+      <c r="C18" s="36">
         <v>1</v>
       </c>
       <c r="D18" s="30" t="s">
@@ -1485,7 +1518,7 @@
     </row>
     <row r="19" spans="1:6" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A19" s="15"/>
-      <c r="B19" s="39" t="s">
+      <c r="B19" s="37" t="s">
         <v>45</v>
       </c>
       <c r="C19" s="29">
@@ -1499,46 +1532,50 @@
     </row>
     <row r="20" spans="1:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="15"/>
-      <c r="B20" s="75" t="s">
-        <v>72</v>
-      </c>
-      <c r="C20" s="58"/>
-      <c r="D20" s="60" t="s">
+      <c r="B20" s="74" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" s="67">
+        <v>0</v>
+      </c>
+      <c r="D20" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="E20" s="62"/>
+      <c r="E20" s="63"/>
       <c r="F20" s="17"/>
     </row>
     <row r="21" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="15"/>
-      <c r="B21" s="76"/>
-      <c r="C21" s="59"/>
-      <c r="D21" s="61"/>
-      <c r="E21" s="63"/>
+      <c r="B21" s="75"/>
+      <c r="C21" s="60"/>
+      <c r="D21" s="62"/>
+      <c r="E21" s="64"/>
       <c r="F21" s="17"/>
     </row>
     <row r="22" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="15"/>
-      <c r="B22" s="41" t="s">
+      <c r="B22" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="42"/>
-      <c r="D22" s="43" t="s">
+      <c r="C22" s="40"/>
+      <c r="D22" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="E22" s="44"/>
+      <c r="E22" s="42"/>
       <c r="F22" s="17"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="15"/>
-      <c r="B23" s="45" t="s">
+      <c r="B23" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="46"/>
-      <c r="D23" s="47" t="s">
+      <c r="C23" s="55">
+        <v>0</v>
+      </c>
+      <c r="D23" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="48"/>
+      <c r="E23" s="45"/>
       <c r="F23" s="17"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1573,72 +1610,72 @@
       <c r="C26" s="29">
         <v>0</v>
       </c>
-      <c r="D26" s="52"/>
+      <c r="D26" s="49"/>
       <c r="E26" s="31"/>
       <c r="F26" s="17"/>
     </row>
     <row r="27" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="15"/>
-      <c r="B27" s="53" t="s">
-        <v>70</v>
+      <c r="B27" s="50" t="s">
+        <v>67</v>
       </c>
       <c r="C27" s="32">
         <v>0</v>
       </c>
-      <c r="D27" s="49"/>
-      <c r="E27" s="40"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="38"/>
       <c r="F27" s="17"/>
     </row>
     <row r="28" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="15"/>
-      <c r="B28" s="53" t="s">
-        <v>71</v>
-      </c>
-      <c r="C28" s="57">
+      <c r="B28" s="50" t="s">
+        <v>68</v>
+      </c>
+      <c r="C28" s="54">
         <v>0</v>
       </c>
-      <c r="D28" s="54"/>
-      <c r="E28" s="55"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="52"/>
       <c r="F28" s="17"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="15"/>
-      <c r="B29" s="50"/>
-      <c r="C29" s="51"/>
+      <c r="B29" s="47"/>
+      <c r="C29" s="48"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="15"/>
-      <c r="B30" s="50"/>
-      <c r="C30" s="51"/>
+      <c r="B30" s="47"/>
+      <c r="C30" s="48"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="15"/>
-      <c r="B31" s="50"/>
+      <c r="B31" s="47"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="15"/>
-      <c r="B32" s="50"/>
+      <c r="B32" s="47"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B33" s="50"/>
+      <c r="B33" s="47"/>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B34" s="50"/>
+      <c r="B34" s="47"/>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B35" s="50"/>
+      <c r="B35" s="47"/>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B36" s="50"/>
+      <c r="B36" s="47"/>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B37" s="50"/>
+      <c r="B37" s="47"/>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B38" s="50"/>
+      <c r="B38" s="47"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A2:A7"/>
     <mergeCell ref="F16:F17"/>
     <mergeCell ref="C20:C21"/>
@@ -1651,6 +1688,7 @@
     <mergeCell ref="C16:C17"/>
     <mergeCell ref="D16:D17"/>
     <mergeCell ref="B20:B21"/>
+    <mergeCell ref="E16:E17"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1697,10 +1735,10 @@
       <c r="B2" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="56">
+      <c r="C2" s="53">
         <v>46183</v>
       </c>
-      <c r="D2" s="52" t="s">
+      <c r="D2" s="49" t="s">
         <v>53</v>
       </c>
       <c r="E2" s="24" t="s">
@@ -1717,10 +1755,10 @@
       <c r="B3" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="56">
+      <c r="C3" s="53">
         <v>46206</v>
       </c>
-      <c r="D3" s="52" t="s">
+      <c r="D3" s="49" t="s">
         <v>53</v>
       </c>
       <c r="E3" s="17" t="s">
@@ -1734,10 +1772,10 @@
       <c r="B4" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="56">
+      <c r="C4" s="53">
         <v>46230</v>
       </c>
-      <c r="D4" s="52" t="s">
+      <c r="D4" s="49" t="s">
         <v>53</v>
       </c>
       <c r="E4" s="26" t="s">
@@ -1777,26 +1815,54 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="17"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="17"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="17"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="17"/>
-      <c r="B9" s="25"/>
+    <row r="7" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="81" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="82">
+        <v>46239</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="81" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="82">
+        <v>46267</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="81" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>74</v>
+      </c>
       <c r="C9" s="17"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="17"/>
+      <c r="D9" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>57</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
chore: Update AI Champions Initiative Report.xlsx with new data
</commit_message>
<xml_diff>
--- a/AI Champions Initiative Report.xlsx
+++ b/AI Champions Initiative Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mpi2cob\Boopathi\Repository\workspace_ai_champion_tracting_dashboard\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mpi2cob\Boopathi\Repository\workspace_ai_champion_tracting_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9DE40A5-80BC-476F-8F62-E135E95F1CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="210" documentId="13_ncr:1_{66A33859-D096-4CB1-8915-ADADD55C98EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31D2F32B-0F09-47A5-8C90-6369B4D2F0F5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D2E0B207-558B-4F0A-AA5E-53ABE0D8DD5B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D2E0B207-558B-4F0A-AA5E-53ABE0D8DD5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet4" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="77">
   <si>
     <t>Initiative Name</t>
   </si>
@@ -57,7 +57,7 @@
     <t>AI Champions Network</t>
   </si>
   <si>
-    <t>Gen AI Champions Initiative@SWD</t>
+    <t>Gen AI Champions Initiative @SWD</t>
   </si>
   <si>
     <t xml:space="preserve">Acharyulu K Karthik (BD/SWD-FSB5)
@@ -118,6 +118,12 @@
     <t>Key Points</t>
   </si>
   <si>
+    <t>Completion Date</t>
+  </si>
+  <si>
+    <t>Docupedia Link</t>
+  </si>
+  <si>
     <t>AI Champions @SWD</t>
   </si>
   <si>
@@ -133,7 +139,8 @@
     <t>ACO - AI Credit Optimizer</t>
   </si>
   <si>
-    <t>Idea shared with BD global</t>
+    <t>Idea shared with BD global
+Phase 2 updates are in-progress</t>
   </si>
   <si>
     <t>BD India Accord Gen AI CoC</t>
@@ -142,120 +149,65 @@
     <t>Benno</t>
   </si>
   <si>
+    <t>Repriortization is going on</t>
+  </si>
+  <si>
     <t>AI Trainings</t>
   </si>
   <si>
-    <t>Langchain, LangGraph</t>
+    <t>Basic of Python, Langchain, LangGraph</t>
   </si>
   <si>
     <t>Claude POC</t>
   </si>
   <si>
+    <t>We dropped POC for Claude LLM since this is already done by other teams.
+Collect input from the team on the feedback of Claude
+Get the information from central team as well</t>
+  </si>
+  <si>
     <t>Sandbox for SWD</t>
   </si>
   <si>
     <t>Its Available</t>
   </si>
   <si>
+    <t>Create a central tracking mechanism (Excel → dashboard/Power BI/JIRA) for all AI activities.</t>
+  </si>
+  <si>
     <t>Boopathi/Nilesh</t>
   </si>
   <si>
+    <t>POCs for Project/Pain points from Buta-Project</t>
+  </si>
+  <si>
+    <t>Possibility to be checked with Srinath and take it forward.
+Personas Profiles</t>
+  </si>
+  <si>
+    <t>Repository - Capture the information - AI topics 
+Gen AI Stories</t>
+  </si>
+  <si>
     <t>Shanthi</t>
   </si>
   <si>
     <t xml:space="preserve">Ideas Usecase - Chatbot </t>
   </si>
   <si>
+    <t>Veeresh - Nilesh</t>
+  </si>
+  <si>
     <t>Calendar for all AI Meets</t>
   </si>
   <si>
     <t>Hackathon</t>
   </si>
   <si>
-    <t>Gen AI Stories</t>
-  </si>
-  <si>
     <t>Gen AI News Letter @SWD</t>
   </si>
   <si>
-    <t>Create a central tracking mechanism (Excel → dashboard/Power BI/JIRA) for all AI activities.</t>
-  </si>
-  <si>
-    <t>Veeresh - Nilesh</t>
-  </si>
-  <si>
-    <t>Sub Topic</t>
-  </si>
-  <si>
-    <t>Session Title</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Owner</t>
-  </si>
-  <si>
-    <t>Link</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>Acharyulu K Karthik</t>
-  </si>
-  <si>
-    <t>DevDock - AI Sandbox for Bosch Developers</t>
-  </si>
-  <si>
-    <t>Building AI-Powered Applications with Spring MCP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Murugaboopathi </t>
-  </si>
-  <si>
-    <t>Sivasankar &amp; Sivasubramanian</t>
-  </si>
-  <si>
-    <t>A2A Protocol in Action: Agent Communication and Workflow Orchestration</t>
-  </si>
-  <si>
-    <t>Upcoming</t>
-  </si>
-  <si>
-    <t>Srilakshmy Sooraj</t>
-  </si>
-  <si>
-    <t>Completion Date</t>
-  </si>
-  <si>
-    <t>Pilot Testing V1</t>
-  </si>
-  <si>
-    <t>V2 Testing</t>
-  </si>
-  <si>
-    <t>https://inside-docupedia.bosch.com/confluence/display/IGPMMCR/System+architecture</t>
-  </si>
-  <si>
-    <t>Phase 2 updates are in-progress</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Define </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>metrics to measure AI benefits (effort savings, productivity).</t>
-    </r>
+    <t>Define metrics to measure AI benefits (effort savings, productivity).</t>
   </si>
   <si>
     <r>
@@ -263,34 +215,79 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Aptos"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> and monthly global connects established.</t>
-    </r>
-  </si>
-  <si>
-    <t>Repository - Capture the information - AI topics Gen AI Stories</t>
-  </si>
-  <si>
-    <t>Repriortization is going on - Sanjeev Sharma will be taking over this topic</t>
-  </si>
-  <si>
-    <r>
-      <t>Collect input from the team on the feedback of Claude, Get the information from central team as well -</t>
+      <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Verdana"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> We are not proceeding with this topic. </t>
+      <t>and monthly global connects established.</t>
     </r>
+  </si>
+  <si>
+    <t>Sub Topic</t>
+  </si>
+  <si>
+    <t>Session Title</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Building AI-Powered Applications with Spring MCP</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Sivasankar &amp; Sivasubramanian</t>
+  </si>
+  <si>
+    <t>https://inside-docupedia.bosch.com/confluence/display/IGPMMCR/System+architecture</t>
+  </si>
+  <si>
+    <t>DevDock - AI Sandbox for Bosch Developers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murugaboopathi </t>
+  </si>
+  <si>
+    <t>A2A Protocol in Action: Agent Communication and Workflow Orchestration</t>
+  </si>
+  <si>
+    <t>Srilakshmy Sooraj</t>
+  </si>
+  <si>
+    <t>Pilot Testing V1</t>
+  </si>
+  <si>
+    <t> </t>
+  </si>
+  <si>
+    <t>Acharyulu K Karthik</t>
+  </si>
+  <si>
+    <t>V2 Testing</t>
+  </si>
+  <si>
+    <t>Upcoming</t>
   </si>
   <si>
     <t>Pilot version</t>
@@ -306,7 +303,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -364,6 +361,12 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -382,16 +385,22 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Verdana"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Verdana"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
       <family val="2"/>
     </font>
     <font>
@@ -399,14 +408,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -441,7 +442,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -643,6 +644,69 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -656,90 +720,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top/>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -748,7 +734,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -797,6 +783,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -809,127 +796,81 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="12" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="12" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="13" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1264,36 +1205,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{651BC675-1C9F-41FC-B0E3-8041898084B3}">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="46.109375" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.5546875" customWidth="1"/>
-    <col min="5" max="5" width="34.44140625" customWidth="1"/>
-    <col min="6" max="6" width="19.77734375" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.109375" customWidth="1"/>
+    <col min="6" max="6" width="19.88671875" customWidth="1"/>
+    <col min="7" max="7" width="18.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="22" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="56" t="s">
+    <row r="2" spans="1:7" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A2" s="58" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="1"/>
@@ -1305,8 +1247,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="56"/>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="58"/>
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1320,8 +1262,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="56"/>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="58"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="2" t="s">
@@ -1331,8 +1273,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="56"/>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="58"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="2" t="s">
@@ -1342,8 +1284,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="56"/>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="58"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2" t="s">
@@ -1353,8 +1295,8 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="57"/>
+    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="59"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="5" t="s">
@@ -1364,8 +1306,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
@@ -1382,315 +1324,263 @@
         <v>24</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="12">
         <f>AVERAGE(C11:C25)</f>
-        <v>0.47272727272727266</v>
+        <v>0.36153846153846148</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="14"/>
       <c r="F10" s="13"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G10" s="13"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="15"/>
       <c r="B11" s="28" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C11" s="29">
         <v>0.5</v>
       </c>
-      <c r="D11" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="27">
-        <v>46387</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D11" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="31"/>
+      <c r="G11" s="16"/>
+    </row>
+    <row r="12" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="15"/>
-      <c r="B12" s="65" t="s">
+      <c r="B12" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="29">
+        <v>0.5</v>
+      </c>
+      <c r="D12" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="67">
+      <c r="E12" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="31"/>
+      <c r="G12" s="16"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="15"/>
+      <c r="B13" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="29">
         <v>0.5</v>
       </c>
-      <c r="D12" s="61" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="F12" s="27"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="15"/>
-      <c r="B13" s="66"/>
-      <c r="C13" s="68"/>
-      <c r="D13" s="69"/>
-      <c r="E13" s="34" t="s">
-        <v>66</v>
-      </c>
-      <c r="F13" s="16"/>
-    </row>
-    <row r="14" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D13" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="31"/>
+      <c r="G13" s="16"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="15"/>
       <c r="B14" s="28" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C14" s="29">
+        <v>0.3</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="31"/>
+      <c r="G14" s="16"/>
+    </row>
+    <row r="15" spans="1:7" ht="76.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="15"/>
+      <c r="B15" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="33">
         <v>1</v>
       </c>
-      <c r="D14" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14" s="76" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="16"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="15"/>
-      <c r="B15" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="29">
-        <v>0.3</v>
-      </c>
-      <c r="D15" s="30" t="s">
+      <c r="D15" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="F15" s="35">
+        <v>46303</v>
+      </c>
+      <c r="G15" s="16"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="15"/>
+      <c r="B16" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="29">
+        <v>1</v>
+      </c>
+      <c r="D16" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" s="31"/>
+      <c r="G16" s="16"/>
+    </row>
+    <row r="17" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="15"/>
+      <c r="B17" s="36" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="29">
+        <v>0.8</v>
+      </c>
+      <c r="D17" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="30"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="16"/>
+    </row>
+    <row r="18" spans="1:7" ht="39" x14ac:dyDescent="0.3">
+      <c r="A18" s="24"/>
+      <c r="B18" s="45" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="46">
+        <v>0.1</v>
+      </c>
+      <c r="D18" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="31" t="s">
+      <c r="E18" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="31"/>
+      <c r="G18" s="16"/>
+    </row>
+    <row r="19" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="24"/>
+      <c r="B19" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="37"/>
+      <c r="D19" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" s="40"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="16"/>
+    </row>
+    <row r="20" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="27"/>
+      <c r="B20" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="29"/>
+      <c r="D20" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="E20" s="30"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="17"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="27"/>
+      <c r="B21" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="29">
+        <v>0</v>
+      </c>
+      <c r="D21" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="F15" s="27"/>
-    </row>
-    <row r="16" spans="1:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="15"/>
-      <c r="B16" s="70" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="77">
-        <v>1</v>
-      </c>
-      <c r="D16" s="72" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" s="79" t="s">
-        <v>71</v>
-      </c>
-      <c r="F16" s="58">
-        <v>46265</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="15"/>
-      <c r="B17" s="71"/>
-      <c r="C17" s="78"/>
-      <c r="D17" s="73"/>
-      <c r="E17" s="80"/>
-      <c r="F17" s="59"/>
-    </row>
-    <row r="18" spans="1:6" ht="27.45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="15"/>
-      <c r="B18" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="36">
-        <v>1</v>
-      </c>
-      <c r="D18" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="E18" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="F18" s="16"/>
-    </row>
-    <row r="19" spans="1:6" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="15"/>
-      <c r="B19" s="37" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" s="29">
-        <v>0.8</v>
-      </c>
-      <c r="D19" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="E19" s="31"/>
-      <c r="F19" s="17"/>
-    </row>
-    <row r="20" spans="1:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="15"/>
-      <c r="B20" s="74" t="s">
-        <v>69</v>
-      </c>
-      <c r="C20" s="67">
+      <c r="E21" s="30"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="17"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="27"/>
+      <c r="B22" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="29">
         <v>0</v>
       </c>
-      <c r="D20" s="61" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="63"/>
-      <c r="F20" s="17"/>
-    </row>
-    <row r="21" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="15"/>
-      <c r="B21" s="75"/>
-      <c r="C21" s="60"/>
-      <c r="D21" s="62"/>
-      <c r="E21" s="64"/>
-      <c r="F21" s="17"/>
-    </row>
-    <row r="22" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="15"/>
-      <c r="B22" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="40"/>
-      <c r="D22" s="41" t="s">
-        <v>46</v>
-      </c>
-      <c r="E22" s="42"/>
-      <c r="F22" s="17"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="15"/>
-      <c r="B23" s="43" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="55">
+      <c r="D22" s="28"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="17"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="17"/>
+      <c r="B23" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="29">
         <v>0</v>
       </c>
-      <c r="D23" s="44" t="s">
-        <v>32</v>
-      </c>
-      <c r="E23" s="45"/>
-      <c r="F23" s="17"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="15"/>
-      <c r="B24" s="35" t="s">
-        <v>42</v>
+      <c r="D23" s="28"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="17"/>
+    </row>
+    <row r="24" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A24" s="17"/>
+      <c r="B24" s="30" t="s">
+        <v>53</v>
       </c>
       <c r="C24" s="29">
         <v>0</v>
       </c>
-      <c r="D24" s="30"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="17"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="15"/>
-      <c r="B25" s="35" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="29">
-        <v>0.1</v>
-      </c>
-      <c r="D25" s="30"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="17"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="15"/>
-      <c r="B26" s="35" t="s">
-        <v>44</v>
-      </c>
-      <c r="C26" s="29">
+      <c r="D24" s="28"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="17"/>
+    </row>
+    <row r="25" spans="1:7" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="18"/>
+      <c r="B25" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="43">
         <v>0</v>
       </c>
-      <c r="D26" s="49"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="17"/>
-    </row>
-    <row r="27" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="15"/>
-      <c r="B27" s="50" t="s">
-        <v>67</v>
-      </c>
-      <c r="C27" s="32">
-        <v>0</v>
-      </c>
-      <c r="D27" s="46"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="17"/>
-    </row>
-    <row r="28" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="15"/>
-      <c r="B28" s="50" t="s">
-        <v>68</v>
-      </c>
-      <c r="C28" s="54">
-        <v>0</v>
-      </c>
-      <c r="D28" s="51"/>
-      <c r="E28" s="52"/>
-      <c r="F28" s="17"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="15"/>
-      <c r="B29" s="47"/>
-      <c r="C29" s="48"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="15"/>
-      <c r="B30" s="47"/>
-      <c r="C30" s="48"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="15"/>
-      <c r="B31" s="47"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="15"/>
-      <c r="B32" s="47"/>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B33" s="47"/>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B34" s="47"/>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B35" s="47"/>
-    </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B36" s="47"/>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B37" s="47"/>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B38" s="47"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="44"/>
+      <c r="G25" s="17"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B26" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="1">
     <mergeCell ref="A2:A7"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="E16:E17"/>
   </mergeCells>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1700,177 +1590,189 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.6640625" customWidth="1"/>
+    <col min="1" max="1" width="27.5546875" customWidth="1"/>
     <col min="2" max="2" width="41.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.77734375" style="23" customWidth="1"/>
+    <col min="3" max="3" width="29.88671875" style="26" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="67.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C1" s="22" t="s">
-        <v>49</v>
+        <v>56</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>57</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="C2" s="53">
+      <c r="A2" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="49">
         <v>46183</v>
       </c>
-      <c r="D2" s="49" t="s">
-        <v>53</v>
-      </c>
-      <c r="E2" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="D2" s="48" t="s">
+        <v>62</v>
+      </c>
+      <c r="E2" s="50" t="s">
+        <v>63</v>
+      </c>
+      <c r="F2" s="51" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="53" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" s="53">
+      <c r="C3" s="54">
         <v>46206</v>
       </c>
-      <c r="D3" s="49" t="s">
-        <v>53</v>
-      </c>
-      <c r="E3" s="17" t="s">
-        <v>57</v>
-      </c>
+      <c r="D3" s="53" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="51"/>
     </row>
     <row r="4" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="C4" s="53">
+      <c r="A4" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="55" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="54">
         <v>46230</v>
       </c>
-      <c r="D4" s="49" t="s">
-        <v>53</v>
-      </c>
-      <c r="E4" s="26" t="s">
-        <v>61</v>
-      </c>
+      <c r="D4" s="53" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="56" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" s="51"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" t="s">
-        <v>65</v>
+      <c r="A5" s="52" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="55" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="53" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="55" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="53" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" s="51" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="E6" s="17" t="s">
-        <v>54</v>
-      </c>
+      <c r="A6" s="52" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="55" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" s="53" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="55" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="53" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" s="51"/>
     </row>
     <row r="7" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="81" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>72</v>
-      </c>
-      <c r="C7" s="82">
+      <c r="A7" s="57" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7" s="54">
         <v>46239</v>
       </c>
-      <c r="D7" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" s="17" t="s">
-        <v>57</v>
-      </c>
+      <c r="D7" s="55" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" s="51"/>
     </row>
     <row r="8" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="81" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="25" t="s">
+      <c r="A8" s="57" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="55" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="54">
+        <v>46267</v>
+      </c>
+      <c r="D8" s="55" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="51"/>
+    </row>
+    <row r="9" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="57" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="55" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" s="53" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="C8" s="82">
-        <v>46267</v>
-      </c>
-      <c r="D8" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="81" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>57</v>
-      </c>
+      <c r="E9" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="F9" s="51"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1 C5:C1048576" xr:uid="{54FEFA70-E4B4-4C12-81BB-70B5E8D78EF0}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1 C10:C1048576" xr:uid="{54FEFA70-E4B4-4C12-81BB-70B5E8D78EF0}">
       <formula1>46023</formula1>
       <formula2>46387</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1 D5:D1048576" xr:uid="{9211E590-0678-4575-A91A-CB6F8551BFC9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1 D10:D1048576" xr:uid="{9211E590-0678-4575-A91A-CB6F8551BFC9}">
       <formula1>"Upcoming, Completed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>